<commit_message>
Almost finished the serializer flow, just need the upload files to be stored in properly named subdirectories
</commit_message>
<xml_diff>
--- a/WorkBot/refactor/data/orders/Ithaca Bakery/Ithaca Bakery_Collegetown_2025-10-08.xlsx
+++ b/WorkBot/refactor/data/orders/Ithaca Bakery/Ithaca Bakery_Collegetown_2025-10-08.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,6 +466,1207 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Monin - Orange</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>8.80</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8.80</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Monin - Butter Pecan</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>9.67</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>67.69</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Monin - Vanilla Sugar Free</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>8.75</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>8.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Monin - Caramel Sugar Free</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>8.75</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>8.75</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WEBSTAURANT</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Monin - Hazelnut</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>8.67</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>17.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Monin - Toffee Nut</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>9.49</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>9.49</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Monin - Peppermint</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Monin - Cookie Butter</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>8.67</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>104.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Caramel Apple Butter</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Monin - Caramel Apple Butter</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>9.25</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>74.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mop Head Cut (White)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Webstaurant</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Container - Soup (16oz)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>5.22</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>20.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lid - Soup (6/16 oz)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>4.82</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>28.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Palmer/Sysco</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Jam - Strawberry</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sysco</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Jelly - Grape</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sysco</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Peanut Butter - Chunky</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>10.22</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>10.22</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>H&amp;M</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Wrap - Foil (9" x 10.75")</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>H&amp;M</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Lid - Portion (3.25oz)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>2.81</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>8.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>H&amp;M/JP</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lid - Portion (2oz)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2.47</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>4.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Monin - Cranberry</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>8.67</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>17.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Hazelnut Coffee (Grounded, Bulk)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>38.00</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>38.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Degreaser - for Panini Press (Dawn)</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>41.16</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>41.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>JadeLeaf</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Matcha - Jade Leaf</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>44.07</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>176.28</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Web/EC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Torani - Caramel Sauce</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Torani - White Chocolate Sauce</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Web/EC</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Torani - Dark Chocolate Sauce</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>H&amp;M</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Cup - Hot (8oz)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LENTZ</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Flax Seeds</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>2.58</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Webstaurant</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Supplement - Whey Protein</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>49.69</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>99.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PKT Salt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>7.92</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>7.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Kilogram Chai Concentrate</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>86.10</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>344.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>vermont</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Maple Syrup (pure)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>42.00</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>42.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Webtaurant</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Container - Deli (16oz)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2.73</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>16.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Java Box (96oz)</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>83.29</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>83.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Java Box (160oz)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>92.59</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>92.59</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Container - Plastic Clamshell (6")</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>FRZ Fruit - Raspberry (Whole)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>FRZ Fruit - Blueberry</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>55.46</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>55.46</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>PALMER</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Bindi - Cake Tiramisu Round</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>32.79</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>32.79</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Palmer</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Sweet Street - Chocolate Lovin</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>45.50</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>45.50</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Grandma's</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Grandma's Coffee Cake - Cinnamon w/ Nuts</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>18.35</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>18.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Grandma's</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Grandma's Coffee Cake - Banana Walnut</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>18.35</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>18.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Grandma's</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Grandma's Coffee Cake - Cranberry</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>18.35</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>18.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Grandma's</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Grandma's Coffee Cake - Pumpkin Spice</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>18.35</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>18.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Palmer</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Sweet Street - Pie Oreo Cookie Bash Sliced</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>PERF</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Vegan Egg</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>99.59</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>99.59</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>BJs</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Chobani - Drinkable Yogurt</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>17.99</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>35.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>BJs</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Celsius - Vibe Peach, Tropical, Arctic</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>28.49</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>28.49</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>